<commit_message>
add workload resize strategy
refactoring

refactoring

refactoring

refactoring

add --resize-strategy parameter

adding resize workload logic

fix test

refactoring

refactoring

add workload resizer

refactoring

add test

add rollback verification logic

add makefile strategy params

add test case

add readme

add readme
</commit_message>
<xml_diff>
--- a/test-env/testbooks/test-cases.xlsx
+++ b/test-env/testbooks/test-cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mariano/Documents/projects/k8s-rightsizer/test-env/testbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A7CB112-3731-674F-A525-5096AF40860E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57275E98-050C-F548-AE69-134AFA545BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Base" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="58">
   <si>
     <t>Namespace</t>
   </si>
@@ -341,6 +341,9 @@
     <t>main-app
 sidecar-1
 sidecar-2</t>
+  </si>
+  <si>
+    <t>test-workload-strategy</t>
   </si>
 </sst>
 </file>
@@ -752,7 +755,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="100" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.83203125" customWidth="1"/>
@@ -1081,6 +1084,33 @@
       <c r="I11" s="9" t="s">
         <v>50</v>
       </c>
+    </row>
+    <row r="12" spans="1:9" ht="100" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="I12" s="14"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>